<commit_message>
SLAM-B modele non concerné par description données
</commit_message>
<xml_diff>
--- a/Data/PGD/PGD_structuration.xlsx
+++ b/Data/PGD/PGD_structuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\PGD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A152AD9B-B756-44EB-BD1C-A87CAC2978B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BFE2A8-6BA5-4F88-ABC2-5FE7217FFBD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{98FDD2D6-D1A3-4DDF-A839-2A0863A95ED3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{98FDD2D6-D1A3-4DDF-A839-2A0863A95ED3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2778" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2944" uniqueCount="622">
   <si>
     <t>Financeur</t>
   </si>
@@ -6314,20 +6314,48 @@
       <c r="AQ14" s="1"/>
       <c r="AR14" s="1"/>
       <c r="AS14" s="1"/>
-      <c r="AT14" s="1"/>
-      <c r="AU14" s="1"/>
-      <c r="AV14" s="1"/>
-      <c r="AW14" s="1"/>
-      <c r="AX14" s="1"/>
-      <c r="AY14" s="1"/>
-      <c r="AZ14" s="1"/>
-      <c r="BA14" s="1"/>
-      <c r="BB14" s="1"/>
-      <c r="BC14" s="1"/>
-      <c r="BD14" s="1"/>
-      <c r="BE14" s="1"/>
-      <c r="BF14" s="1"/>
-      <c r="BG14" s="1"/>
+      <c r="AT14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF14" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG14" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH14" s="1"/>
       <c r="BI14" s="1"/>
       <c r="BJ14" s="1"/>
@@ -6501,20 +6529,48 @@
       <c r="AQ15" s="1"/>
       <c r="AR15" s="1"/>
       <c r="AS15" s="1"/>
-      <c r="AT15" s="1"/>
-      <c r="AU15" s="1"/>
-      <c r="AV15" s="1"/>
-      <c r="AW15" s="1"/>
-      <c r="AX15" s="1"/>
-      <c r="AY15" s="1"/>
-      <c r="AZ15" s="1"/>
-      <c r="BA15" s="1"/>
-      <c r="BB15" s="1"/>
-      <c r="BC15" s="1"/>
-      <c r="BD15" s="1"/>
-      <c r="BE15" s="1"/>
-      <c r="BF15" s="1"/>
-      <c r="BG15" s="1"/>
+      <c r="AT15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF15" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG15" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH15" s="1"/>
       <c r="BI15" s="1"/>
       <c r="BJ15" s="1"/>
@@ -6875,20 +6931,48 @@
       <c r="AQ17" s="1"/>
       <c r="AR17" s="1"/>
       <c r="AS17" s="1"/>
-      <c r="AT17" s="1"/>
-      <c r="AU17" s="1"/>
-      <c r="AV17" s="1"/>
-      <c r="AW17" s="1"/>
-      <c r="AX17" s="1"/>
-      <c r="AY17" s="1"/>
-      <c r="AZ17" s="1"/>
-      <c r="BA17" s="1"/>
-      <c r="BB17" s="1"/>
-      <c r="BC17" s="1"/>
-      <c r="BD17" s="1"/>
-      <c r="BE17" s="1"/>
-      <c r="BF17" s="1"/>
-      <c r="BG17" s="1"/>
+      <c r="AT17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF17" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG17" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH17" s="1"/>
       <c r="BI17" s="1"/>
       <c r="BJ17" s="1"/>
@@ -7062,20 +7146,48 @@
       <c r="AQ18" s="1"/>
       <c r="AR18" s="1"/>
       <c r="AS18" s="1"/>
-      <c r="AT18" s="1"/>
-      <c r="AU18" s="1"/>
-      <c r="AV18" s="1"/>
-      <c r="AW18" s="1"/>
-      <c r="AX18" s="1"/>
-      <c r="AY18" s="1"/>
-      <c r="AZ18" s="1"/>
-      <c r="BA18" s="1"/>
-      <c r="BB18" s="1"/>
-      <c r="BC18" s="1"/>
-      <c r="BD18" s="1"/>
-      <c r="BE18" s="1"/>
-      <c r="BF18" s="1"/>
-      <c r="BG18" s="1"/>
+      <c r="AT18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF18" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG18" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH18" s="1"/>
       <c r="BI18" s="1"/>
       <c r="BJ18" s="1"/>
@@ -7249,20 +7361,48 @@
       <c r="AQ19" s="1"/>
       <c r="AR19" s="1"/>
       <c r="AS19" s="1"/>
-      <c r="AT19" s="1"/>
-      <c r="AU19" s="1"/>
-      <c r="AV19" s="1"/>
-      <c r="AW19" s="1"/>
-      <c r="AX19" s="1"/>
-      <c r="AY19" s="1"/>
-      <c r="AZ19" s="1"/>
-      <c r="BA19" s="1"/>
-      <c r="BB19" s="1"/>
-      <c r="BC19" s="1"/>
-      <c r="BD19" s="1"/>
-      <c r="BE19" s="1"/>
-      <c r="BF19" s="1"/>
-      <c r="BG19" s="1"/>
+      <c r="AT19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF19" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG19" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH19" s="1"/>
       <c r="BI19" s="1"/>
       <c r="BJ19" s="1"/>
@@ -7436,20 +7576,48 @@
       <c r="AQ20" s="1"/>
       <c r="AR20" s="1"/>
       <c r="AS20" s="1"/>
-      <c r="AT20" s="1"/>
-      <c r="AU20" s="1"/>
-      <c r="AV20" s="1"/>
-      <c r="AW20" s="1"/>
-      <c r="AX20" s="1"/>
-      <c r="AY20" s="1"/>
-      <c r="AZ20" s="1"/>
-      <c r="BA20" s="1"/>
-      <c r="BB20" s="1"/>
-      <c r="BC20" s="1"/>
-      <c r="BD20" s="1"/>
-      <c r="BE20" s="1"/>
-      <c r="BF20" s="1"/>
-      <c r="BG20" s="1"/>
+      <c r="AT20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF20" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG20" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH20" s="1"/>
       <c r="BI20" s="1"/>
       <c r="BJ20" s="1"/>
@@ -7623,20 +7791,48 @@
       <c r="AQ21" s="1"/>
       <c r="AR21" s="1"/>
       <c r="AS21" s="1"/>
-      <c r="AT21" s="1"/>
-      <c r="AU21" s="1"/>
-      <c r="AV21" s="1"/>
-      <c r="AW21" s="1"/>
-      <c r="AX21" s="1"/>
-      <c r="AY21" s="1"/>
-      <c r="AZ21" s="1"/>
-      <c r="BA21" s="1"/>
-      <c r="BB21" s="1"/>
-      <c r="BC21" s="1"/>
-      <c r="BD21" s="1"/>
-      <c r="BE21" s="1"/>
-      <c r="BF21" s="1"/>
-      <c r="BG21" s="1"/>
+      <c r="AT21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF21" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG21" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH21" s="1"/>
       <c r="BI21" s="1"/>
       <c r="BJ21" s="1"/>
@@ -7810,20 +8006,48 @@
       <c r="AQ22" s="1"/>
       <c r="AR22" s="1"/>
       <c r="AS22" s="1"/>
-      <c r="AT22" s="1"/>
-      <c r="AU22" s="1"/>
-      <c r="AV22" s="1"/>
-      <c r="AW22" s="1"/>
-      <c r="AX22" s="1"/>
-      <c r="AY22" s="1"/>
-      <c r="AZ22" s="1"/>
-      <c r="BA22" s="1"/>
-      <c r="BB22" s="1"/>
-      <c r="BC22" s="1"/>
-      <c r="BD22" s="1"/>
-      <c r="BE22" s="1"/>
-      <c r="BF22" s="1"/>
-      <c r="BG22" s="1"/>
+      <c r="AT22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF22" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG22" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH22" s="1"/>
       <c r="BI22" s="1"/>
       <c r="BJ22" s="1"/>
@@ -7997,20 +8221,48 @@
       <c r="AQ23" s="1"/>
       <c r="AR23" s="1"/>
       <c r="AS23" s="1"/>
-      <c r="AT23" s="1"/>
-      <c r="AU23" s="1"/>
-      <c r="AV23" s="1"/>
-      <c r="AW23" s="1"/>
-      <c r="AX23" s="1"/>
-      <c r="AY23" s="1"/>
-      <c r="AZ23" s="1"/>
-      <c r="BA23" s="1"/>
-      <c r="BB23" s="1"/>
-      <c r="BC23" s="1"/>
-      <c r="BD23" s="1"/>
-      <c r="BE23" s="1"/>
-      <c r="BF23" s="1"/>
-      <c r="BG23" s="1"/>
+      <c r="AT23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF23" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG23" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH23" s="1"/>
       <c r="BI23" s="1"/>
       <c r="BJ23" s="1"/>
@@ -8184,20 +8436,48 @@
       <c r="AQ24" s="1"/>
       <c r="AR24" s="1"/>
       <c r="AS24" s="1"/>
-      <c r="AT24" s="1"/>
-      <c r="AU24" s="1"/>
-      <c r="AV24" s="1"/>
-      <c r="AW24" s="1"/>
-      <c r="AX24" s="1"/>
-      <c r="AY24" s="1"/>
-      <c r="AZ24" s="1"/>
-      <c r="BA24" s="1"/>
-      <c r="BB24" s="1"/>
-      <c r="BC24" s="1"/>
-      <c r="BD24" s="1"/>
-      <c r="BE24" s="1"/>
-      <c r="BF24" s="1"/>
-      <c r="BG24" s="1"/>
+      <c r="AT24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF24" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG24" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH24" s="1"/>
       <c r="BI24" s="1"/>
       <c r="BJ24" s="1"/>
@@ -8371,24 +8651,48 @@
       <c r="AQ25" s="1"/>
       <c r="AR25" s="1"/>
       <c r="AS25" s="1"/>
-      <c r="AT25" s="1"/>
-      <c r="AU25" s="1"/>
-      <c r="AV25" s="1"/>
-      <c r="AW25" s="1"/>
-      <c r="AX25" s="1"/>
-      <c r="AY25" s="1"/>
-      <c r="AZ25" s="1"/>
+      <c r="AT25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ25" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BA25" s="1" t="s">
         <v>573</v>
       </c>
       <c r="BB25" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="BC25" s="1"/>
-      <c r="BD25" s="1"/>
-      <c r="BE25" s="1"/>
-      <c r="BF25" s="1"/>
-      <c r="BG25" s="1"/>
+      <c r="BC25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF25" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG25" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH25" s="1" t="s">
         <v>578</v>
       </c>
@@ -10719,20 +11023,48 @@
       <c r="AQ37" s="1"/>
       <c r="AR37" s="1"/>
       <c r="AS37" s="1"/>
-      <c r="AT37" s="1"/>
-      <c r="AU37" s="1"/>
-      <c r="AV37" s="1"/>
-      <c r="AW37" s="1"/>
-      <c r="AX37" s="1"/>
-      <c r="AY37" s="1"/>
-      <c r="AZ37" s="1"/>
-      <c r="BA37" s="1"/>
-      <c r="BB37" s="1"/>
-      <c r="BC37" s="1"/>
-      <c r="BD37" s="1"/>
-      <c r="BE37" s="1"/>
-      <c r="BF37" s="1"/>
-      <c r="BG37" s="1"/>
+      <c r="AT37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AU37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AV37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AW37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AX37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AY37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="AZ37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BA37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BB37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BC37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BD37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BE37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BF37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="BG37" s="1" t="s">
+        <v>450</v>
+      </c>
       <c r="BH37" s="1"/>
       <c r="BI37" s="1"/>
       <c r="BJ37" s="1"/>

</xml_diff>

<commit_message>
ajout fichier de base
</commit_message>
<xml_diff>
--- a/Data/PGD/PGD_structuration.xlsx
+++ b/Data/PGD/PGD_structuration.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\PGD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844B42F7-CB3C-4D1F-A2E5-4B96D28D1FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07CE63ED-F687-4B89-A96A-A83945911CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{98FDD2D6-D1A3-4DDF-A839-2A0863A95ED3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{98FDD2D6-D1A3-4DDF-A839-2A0863A95ED3}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$CP$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$CP$84</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2984" uniqueCount="1052">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2986" uniqueCount="1053">
   <si>
     <t>Financeur</t>
   </si>
@@ -5080,6 +5080,9 @@
 GAMS licence is needed to change the codes and run the models.
 Statistical software such as Stata or R will be used for analysing survey data. No licence is required for R (free software);
 however, Stata licence is needed to change the code and execute the model.</t>
+  </si>
+  <si>
+    <t>&amp;questions&amp;</t>
   </si>
 </sst>
 </file>
@@ -21043,8 +21046,12 @@
       </c>
     </row>
     <row r="80" spans="1:102" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A80" s="22"/>
-      <c r="B80" s="22"/>
+      <c r="A80" s="22" t="s">
+        <v>396</v>
+      </c>
+      <c r="B80" s="22" t="s">
+        <v>1052</v>
+      </c>
       <c r="C80" s="23"/>
       <c r="D80" s="22"/>
       <c r="E80" s="22" t="s">
@@ -21911,7 +21918,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CP1" xr:uid="{E04D9850-7CF0-4E84-8E6E-B467C0834BD4}"/>
+  <autoFilter ref="A1:CP84" xr:uid="{E04D9850-7CF0-4E84-8E6E-B467C0834BD4}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="E3 E14 E42 E57 E52:E54 E71 E63 E65 E61 E80:E83">
     <cfRule type="containsText" dxfId="109" priority="122" operator="containsText" text="INSUFFISANT">

</xml_diff>